<commit_message>
0.85 - forms alignment
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\pets-and-maintenance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1A4A068-3C02-482F-BEB6-98425F8E3AD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F30DE2C-FAFB-4EAF-B68B-4EC8F605FF9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="17070" yWindow="0" windowWidth="11835" windowHeight="15585" activeTab="1" xr2:uid="{940A306A-87ED-4B7D-95ED-E3380541153A}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="107">
   <si>
     <t>מזהה (ID)</t>
   </si>
@@ -356,6 +356,15 @@
   </si>
   <si>
     <t>חווית ONBORDING למשתמש</t>
+  </si>
+  <si>
+    <t>חיווי תאריך ביצעו אחרון של משימה</t>
+  </si>
+  <si>
+    <t>תיקון כפתור הפלוס וכפתור העריכה שפותחים טופס לא מותאם לקבוצות ופריטים בהגדרות</t>
+  </si>
+  <si>
+    <t>טקסט דינמי בחלונית עריכת משימה</t>
   </si>
 </sst>
 </file>
@@ -1134,7 +1143,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE9D0107-5AD1-4C19-82D2-5754FE2AF02D}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr defaultColWidth="57" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.125" bestFit="1" customWidth="1"/>
@@ -1217,7 +1226,7 @@
         <v>66</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>57</v>
@@ -1584,6 +1593,24 @@
       </c>
       <c r="E27" s="7" t="s">
         <v>103</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B28" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E28" s="7" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="E29" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E30" s="7" t="s">
+        <v>106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>